<commit_message>
refactor(core): improve encoding handling, keyword matching, and cleanup debug files
- Refactor main.py: add mojibake-resistant log reading (read_log_text), OS version comparison, and log keyword extraction
- Refactor compare.py: extract KEYWORD_MAPPING to class constant, add _normalize_keyword for fuzzy matching (case/space/get-prefix insensitive), enable alias-based lookup across log and web sources
- Clean up debug/test/scratch files (audit pages, debug scripts, screenshots, old logs)
- Remove __pycache__ from tracking
- Add README.md, data/log.txt, data/test.txt
- Update checklist.xlsx and result.xlsx data
</commit_message>
<xml_diff>
--- a/ai_checker/data/checklist.xlsx
+++ b/ai_checker/data/checklist.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="25920" windowHeight="12300" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="28800" windowHeight="12300" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="checklist" sheetId="1" state="visible" r:id="rId1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="35">
+  <fonts count="32">
     <font>
       <name val="宋体"/>
       <charset val="134"/>
@@ -243,26 +243,6 @@
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="微软雅黑"/>
-      <charset val="134"/>
-      <b val="1"/>
-      <color theme="5"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <name val="微软雅黑"/>
-      <charset val="134"/>
-      <b val="1"/>
-      <color theme="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="微软雅黑"/>
-      <charset val="134"/>
-      <color rgb="FFFF0000"/>
-      <sz val="12"/>
     </font>
   </fonts>
   <fills count="40">
@@ -598,7 +578,9 @@
         <color auto="1"/>
       </right>
       <top/>
-      <bottom/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -609,9 +591,7 @@
         <color auto="1"/>
       </right>
       <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -872,10 +852,11 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="6">
       <alignment vertical="center"/>
     </xf>
@@ -909,15 +890,10 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -930,12 +906,8 @@
     <xf numFmtId="0" fontId="8" fillId="5" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -966,24 +938,15 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="49">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="49">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="49">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -999,24 +962,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1026,10 +980,6 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="50">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1084,7 +1034,74 @@
     <cellStyle name="RowLevel_8 3" xfId="49"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -1381,24 +1398,24 @@
   <dimension ref="A1:H32"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="17.4"/>
   <cols>
-    <col width="16.7314814814815" customWidth="1" style="51" min="2" max="2"/>
-    <col width="33.462962962963" customWidth="1" style="51" min="3" max="3"/>
-    <col width="9.861111111111111" customWidth="1" style="51" min="4" max="4"/>
-    <col width="71.60185185185181" customWidth="1" style="51" min="5" max="5"/>
-    <col width="28.6018518518519" customWidth="1" style="51" min="6" max="6"/>
-    <col width="29.1296296296296" customWidth="1" style="51" min="7" max="7"/>
-    <col width="60.2685185185185" customWidth="1" style="11" min="8" max="8"/>
+    <col width="16.7314814814815" customWidth="1" style="1" min="2" max="2"/>
+    <col width="33.462962962963" customWidth="1" style="1" min="3" max="3"/>
+    <col width="9.861111111111111" customWidth="1" style="1" min="4" max="4"/>
+    <col width="71.60185185185181" customWidth="1" style="1" min="5" max="5"/>
+    <col width="28.6018518518519" customWidth="1" style="1" min="6" max="6"/>
+    <col width="29.1296296296296" customWidth="1" style="1" min="7" max="7"/>
+    <col width="60.2685185185185" customWidth="1" style="12" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="33.75" customHeight="1" s="51">
+    <row r="1" ht="33.75" customHeight="1" s="1">
       <c r="A1" s="13" t="inlineStr">
         <is>
           <t>OpenHarmony生态产品兼容性测评评估Checklist--商用设备</t>
         </is>
       </c>
-      <c r="G1" s="52" t="n"/>
-    </row>
-    <row r="2" ht="81.75" customHeight="1" s="51">
+      <c r="G1" s="14" t="n"/>
+    </row>
+    <row r="2" ht="81.75" customHeight="1" s="1">
       <c r="A2" s="15" t="inlineStr">
         <is>
           <t>适用场景：
@@ -1407,7 +1424,7 @@
 3、其他场景请咨询兼容性工作组，解释权归工作组团队所有。</t>
         </is>
       </c>
-      <c r="G2" s="52" t="n"/>
+      <c r="G2" s="14" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="16" t="inlineStr">
@@ -1446,12 +1463,12 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="52.2" customHeight="1" s="51">
-      <c r="A4" s="53" t="n"/>
-      <c r="B4" s="54" t="n"/>
-      <c r="C4" s="53" t="n"/>
-      <c r="D4" s="53" t="n"/>
-      <c r="E4" s="53" t="n"/>
+    <row r="4" ht="52.2" customHeight="1" s="1">
+      <c r="A4" s="19" t="n"/>
+      <c r="B4" s="20" t="n"/>
+      <c r="C4" s="19" t="n"/>
+      <c r="D4" s="19" t="n"/>
+      <c r="E4" s="19" t="n"/>
       <c r="F4" s="21" t="inlineStr">
         <is>
           <t>填写结果√（满足）， ×（不满足）， NA（不涉及）</t>
@@ -1469,7 +1486,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="174" customHeight="1" s="51">
+    <row r="5" ht="174" customHeight="1" s="1">
       <c r="A5" s="24" t="n">
         <v>1</v>
       </c>
@@ -1499,7 +1516,7 @@
       </c>
       <c r="F5" s="29" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✔</t>
         </is>
       </c>
       <c r="G5" s="21" t="n"/>
@@ -1510,7 +1527,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="52.2" customHeight="1" s="51">
+    <row r="6" ht="52.2" customHeight="1" s="1">
       <c r="A6" s="24" t="n">
         <v>2</v>
       </c>
@@ -1537,18 +1554,18 @@
       </c>
       <c r="F6" s="29" t="n"/>
       <c r="G6" s="21" t="n"/>
-      <c r="H6" s="32" t="inlineStr">
+      <c r="H6" s="31" t="inlineStr">
         <is>
           <t>若测评中未提供，无法烧录，应驳回厂商修改补充。
 驳回话术参考：材料缺失，缺少烧录的软件工具及烧录指导，需提供。</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="49.8" customHeight="1" s="51">
+    <row r="7" ht="49.8" customHeight="1" s="1">
       <c r="A7" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="54" t="n"/>
+      <c r="B7" s="20" t="n"/>
       <c r="C7" s="26" t="inlineStr">
         <is>
           <t>固件/镜像文件包
@@ -1567,20 +1584,20 @@
       </c>
       <c r="F7" s="29" t="n"/>
       <c r="G7" s="21" t="n"/>
-      <c r="H7" s="34" t="n"/>
-    </row>
-    <row r="8" ht="80" customHeight="1" s="51">
+      <c r="H7" s="32" t="n"/>
+    </row>
+    <row r="8" ht="80" customHeight="1" s="1">
       <c r="A8" s="24" t="n">
         <v>4</v>
       </c>
-      <c r="B8" s="54" t="n"/>
+      <c r="B8" s="20" t="n"/>
       <c r="C8" s="26" t="inlineStr">
         <is>
           <t>测试套件
 （所在位置：测评中，报告上传-镜像文件或XTS报告）</t>
         </is>
       </c>
-      <c r="D8" s="35" t="inlineStr">
+      <c r="D8" s="33" t="inlineStr">
         <is>
           <t>非必选</t>
         </is>
@@ -1592,18 +1609,18 @@
       </c>
       <c r="F8" s="29" t="n"/>
       <c r="G8" s="21" t="n"/>
-      <c r="H8" s="32" t="inlineStr">
+      <c r="H8" s="31" t="inlineStr">
         <is>
           <t>若非arm32未提供，无法测试，应驳回厂商提供。
 驳回话术参考：材料缺失，缺少XTS测试套件，需提供。</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="140" customHeight="1" s="51">
+    <row r="9" ht="140" customHeight="1" s="1">
       <c r="A9" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="53" t="n"/>
+      <c r="B9" s="19" t="n"/>
       <c r="C9" s="26" t="inlineStr">
         <is>
           <t>可视化测试报告或测试日志
@@ -1624,7 +1641,7 @@
       </c>
       <c r="F9" s="29" t="n"/>
       <c r="G9" s="21" t="n"/>
-      <c r="H9" s="32" t="inlineStr">
+      <c r="H9" s="31" t="inlineStr">
         <is>
           <t>若提供的XTS报告存在失败项未处理、缺少部分最小集报告、豁免申请与测评中XTS报告失败项不一致等情况，应驳回至厂商。
 驳回话术参考：1、SSTS材料缺失，缺少部分模块执行结果，需提供测试通过的可视化报告或进行豁免申请。
@@ -1632,7 +1649,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="104.4" customHeight="1" s="51">
+    <row r="10" ht="104.4" customHeight="1" s="1">
       <c r="A10" s="24" t="n">
         <v>6</v>
       </c>
@@ -1641,7 +1658,7 @@
           <t>PCS（产品兼容性技术规范文档）</t>
         </is>
       </c>
-      <c r="C10" s="37" t="inlineStr">
+      <c r="C10" s="34" t="inlineStr">
         <is>
           <t>OpenHarmony设备兼容性规范自检表（所在位置：测评中，报告上传-PCS自检表）</t>
         </is>
@@ -1651,7 +1668,7 @@
           <t>必选要求</t>
         </is>
       </c>
-      <c r="E10" s="38" t="inlineStr">
+      <c r="E10" s="35" t="inlineStr">
         <is>
           <t>1、提供的PCS自检表需使用对应版本、对应系统类型的PCS
 2、E列自检结果需填写完整
@@ -1661,7 +1678,7 @@
       </c>
       <c r="F10" s="29" t="n"/>
       <c r="G10" s="21" t="n"/>
-      <c r="H10" s="32" t="inlineStr">
+      <c r="H10" s="31" t="inlineStr">
         <is>
           <t>不符合要求项，应进行驳回处理
 驳回话术参考：1、PCS自检表第97-99行E列自检结果标N项未在F列备注说明原因，需修改。
@@ -1669,16 +1686,16 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="147" customHeight="1" s="51">
+    <row r="11" ht="147" customHeight="1" s="1">
       <c r="A11" s="24" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="39" t="inlineStr">
+      <c r="B11" s="36" t="inlineStr">
         <is>
           <t>测评XTS豁免申请核对</t>
         </is>
       </c>
-      <c r="C11" s="39" t="inlineStr">
+      <c r="C11" s="36" t="inlineStr">
         <is>
           <t>豁免问题核对（所在位置：测评中，测评豁免申请）</t>
         </is>
@@ -1688,7 +1705,7 @@
           <t>必选要求</t>
         </is>
       </c>
-      <c r="E11" s="40" t="inlineStr">
+      <c r="E11" s="37" t="inlineStr">
         <is>
           <t>1、检查豁免申请填写是否符合要求；
 --模块名称，仅可输入一个；
@@ -1700,8 +1717,8 @@
         </is>
       </c>
       <c r="F11" s="29" t="n"/>
-      <c r="G11" s="41" t="n"/>
-      <c r="H11" s="32" t="inlineStr">
+      <c r="G11" s="38" t="n"/>
+      <c r="H11" s="31" t="inlineStr">
         <is>
           <t>不符合要求项，应进行驳回处理
 驳回话术参考：1、xxx模块的xx测试套存在豁免失败，需处理。
@@ -1709,7 +1726,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="34.8" customHeight="1" s="51">
+    <row r="12" ht="34.8" customHeight="1" s="1">
       <c r="A12" s="24" t="n">
         <v>8</v>
       </c>
@@ -1723,7 +1740,7 @@
           <t>企业全称（英文）</t>
         </is>
       </c>
-      <c r="D12" s="35" t="inlineStr">
+      <c r="D12" s="33" t="inlineStr">
         <is>
           <t>非必选</t>
         </is>
@@ -1735,19 +1752,19 @@
       </c>
       <c r="F12" s="29" t="n"/>
       <c r="G12" s="21" t="n"/>
-      <c r="H12" s="34" t="n"/>
-    </row>
-    <row r="13" ht="34.8" customHeight="1" s="51">
+      <c r="H12" s="32" t="n"/>
+    </row>
+    <row r="13" ht="34.8" customHeight="1" s="1">
       <c r="A13" s="24" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="54" t="n"/>
+      <c r="B13" s="20" t="n"/>
       <c r="C13" s="26" t="inlineStr">
         <is>
           <t>企业简称</t>
         </is>
       </c>
-      <c r="D13" s="35" t="inlineStr">
+      <c r="D13" s="33" t="inlineStr">
         <is>
           <t>非必选</t>
         </is>
@@ -1759,13 +1776,13 @@
       </c>
       <c r="F13" s="29" t="n"/>
       <c r="G13" s="21" t="n"/>
-      <c r="H13" s="34" t="n"/>
-    </row>
-    <row r="14" ht="52.2" customHeight="1" s="51">
+      <c r="H13" s="32" t="n"/>
+    </row>
+    <row r="14" ht="52.2" customHeight="1" s="1">
       <c r="A14" s="24" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="53" t="n"/>
+      <c r="B14" s="19" t="n"/>
       <c r="C14" s="26" t="inlineStr">
         <is>
           <t>企业简称（英文）</t>
@@ -1784,13 +1801,13 @@
       </c>
       <c r="F14" s="29" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✔</t>
         </is>
       </c>
       <c r="G14" s="21" t="n"/>
-      <c r="H14" s="34" t="n"/>
-    </row>
-    <row r="15" ht="42" customHeight="1" s="51">
+      <c r="H14" s="32" t="n"/>
+    </row>
+    <row r="15" ht="42" customHeight="1" s="1">
       <c r="A15" s="24" t="n">
         <v>11</v>
       </c>
@@ -1799,7 +1816,7 @@
           <t>产品定义/软件定义</t>
         </is>
       </c>
-      <c r="C15" s="37" t="inlineStr">
+      <c r="C15" s="34" t="inlineStr">
         <is>
           <t>测评类型</t>
         </is>
@@ -1809,21 +1826,21 @@
           <t>必选要求</t>
         </is>
       </c>
-      <c r="E15" s="43" t="inlineStr">
+      <c r="E15" s="39" t="inlineStr">
         <is>
           <t>根据外观图、实际投递样机产品外观结构，判断是否与模组/开发板、商用设备、软件发行版测评类型相符</t>
         </is>
       </c>
       <c r="F15" s="29" t="n"/>
       <c r="G15" s="21" t="n"/>
-      <c r="H15" s="34" t="n"/>
-    </row>
-    <row r="16" ht="34.8" customHeight="1" s="51">
+      <c r="H15" s="32" t="n"/>
+    </row>
+    <row r="16" ht="34.8" customHeight="1" s="1">
       <c r="A16" s="24" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="54" t="n"/>
-      <c r="C16" s="37" t="inlineStr">
+      <c r="B16" s="20" t="n"/>
+      <c r="C16" s="34" t="inlineStr">
         <is>
           <t>操作系统类型</t>
         </is>
@@ -1833,21 +1850,21 @@
           <t>必选要求</t>
         </is>
       </c>
-      <c r="E16" s="43" t="inlineStr">
+      <c r="E16" s="39" t="inlineStr">
         <is>
           <t>根据芯片、镜像、XTS测试报告，判断是否与轻量系统、小型系统、标准系统OS类型相符</t>
         </is>
       </c>
       <c r="F16" s="29" t="n"/>
       <c r="G16" s="21" t="n"/>
-      <c r="H16" s="34" t="n"/>
-    </row>
-    <row r="17" ht="104.4" customHeight="1" s="51">
+      <c r="H16" s="32" t="n"/>
+    </row>
+    <row r="17" ht="104.4" customHeight="1" s="1">
       <c r="A17" s="24" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="54" t="n"/>
-      <c r="C17" s="45" t="inlineStr">
+      <c r="B17" s="20" t="n"/>
+      <c r="C17" s="40" t="inlineStr">
         <is>
           <t>操作系统版本号</t>
         </is>
@@ -1857,7 +1874,7 @@
           <t>必选要求</t>
         </is>
       </c>
-      <c r="E17" s="43" t="inlineStr">
+      <c r="E17" s="39" t="inlineStr">
         <is>
           <t>1、检查操作系统版本号前两位版本号与设备侧固件包读取的GetOsFullName()前两位是否一致；
 2、检查设备侧读取的GetOsFullName()与xts报告中OsFullName是否一致，
@@ -1866,18 +1883,18 @@
       </c>
       <c r="F17" s="29" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✔</t>
         </is>
       </c>
       <c r="G17" s="21" t="n"/>
-      <c r="H17" s="34" t="n"/>
-    </row>
-    <row r="18" ht="121.8" customHeight="1" s="51">
+      <c r="H17" s="32" t="n"/>
+    </row>
+    <row r="18" ht="121.8" customHeight="1" s="1">
       <c r="A18" s="24" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="54" t="n"/>
-      <c r="C18" s="45" t="inlineStr">
+      <c r="B18" s="20" t="n"/>
+      <c r="C18" s="40" t="inlineStr">
         <is>
           <t>设备名称（传播名）</t>
         </is>
@@ -1887,7 +1904,7 @@
           <t>必选要求</t>
         </is>
       </c>
-      <c r="E18" s="43" t="inlineStr">
+      <c r="E18" s="39" t="inlineStr">
         <is>
           <t>1、首次提交时间在2026.02.09及之后的测评审核时，
 设备侧GetMarketName()、XTS报告中MarketName、测评中填写的传播名保持一致即可，字符长度、语种均不审视。
@@ -1896,18 +1913,18 @@
       </c>
       <c r="F18" s="29" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✔</t>
         </is>
       </c>
       <c r="G18" s="21" t="n"/>
-      <c r="H18" s="34" t="n"/>
-    </row>
-    <row r="19" ht="52.2" customHeight="1" s="51">
+      <c r="H18" s="32" t="n"/>
+    </row>
+    <row r="19" ht="52.2" customHeight="1" s="1">
       <c r="A19" s="24" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="54" t="n"/>
-      <c r="C19" s="45" t="inlineStr">
+      <c r="B19" s="20" t="n"/>
+      <c r="C19" s="40" t="inlineStr">
         <is>
           <t>设备型号</t>
         </is>
@@ -1917,7 +1934,7 @@
           <t>必选要求</t>
         </is>
       </c>
-      <c r="E19" s="43" t="inlineStr">
+      <c r="E19" s="39" t="inlineStr">
         <is>
           <t>1、需要采用英文描述，最多32字符。
 2、测评中设备型号、设备侧读取GetProductModel()、XTS报告中ProductModel需保持一致</t>
@@ -1925,18 +1942,18 @@
       </c>
       <c r="F19" s="29" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✔</t>
         </is>
       </c>
       <c r="G19" s="21" t="n"/>
-      <c r="H19" s="34" t="n"/>
-    </row>
-    <row r="20" ht="69.59999999999999" customHeight="1" s="51">
+      <c r="H19" s="32" t="n"/>
+    </row>
+    <row r="20" ht="69.59999999999999" customHeight="1" s="1">
       <c r="A20" s="24" t="n">
         <v>16</v>
       </c>
-      <c r="B20" s="54" t="n"/>
-      <c r="C20" s="45" t="inlineStr">
+      <c r="B20" s="20" t="n"/>
+      <c r="C20" s="40" t="inlineStr">
         <is>
           <t>设备类型</t>
         </is>
@@ -1946,7 +1963,7 @@
           <t>必选要求</t>
         </is>
       </c>
-      <c r="E20" s="43" t="inlineStr">
+      <c r="E20" s="39" t="inlineStr">
         <is>
           <t>1、GetDeviceType()设备类型，最多32个字符，不允许使用中文。
 2、测评中的版本id首个字段、设备侧读取GetDeviceType()、XTS报告中DeviceType需保持一致（测评中产品定义-设备类型无需审核）
@@ -1955,14 +1972,14 @@
       </c>
       <c r="F20" s="29" t="n"/>
       <c r="G20" s="21" t="n"/>
-      <c r="H20" s="34" t="n"/>
-    </row>
-    <row r="21" ht="52.2" customHeight="1" s="51">
+      <c r="H20" s="32" t="n"/>
+    </row>
+    <row r="21" ht="52.2" customHeight="1" s="1">
       <c r="A21" s="24" t="n">
         <v>17</v>
       </c>
-      <c r="B21" s="54" t="n"/>
-      <c r="C21" s="45" t="inlineStr">
+      <c r="B21" s="20" t="n"/>
+      <c r="C21" s="40" t="inlineStr">
         <is>
           <t>品牌英文名称</t>
         </is>
@@ -1972,7 +1989,7 @@
           <t>必选要求</t>
         </is>
       </c>
-      <c r="E21" s="43" t="inlineStr">
+      <c r="E21" s="39" t="inlineStr">
         <is>
           <t>1、品牌英文名称，最多32字符。
 2、测评中品牌英文名称、设备侧读取GetBrand()、XTS报告中Brand需保持一致</t>
@@ -1980,18 +1997,18 @@
       </c>
       <c r="F21" s="29" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✔</t>
         </is>
       </c>
       <c r="G21" s="21" t="n"/>
-      <c r="H21" s="34" t="n"/>
-    </row>
-    <row r="22" ht="75" customHeight="1" s="51">
+      <c r="H21" s="32" t="n"/>
+    </row>
+    <row r="22" ht="75" customHeight="1" s="1">
       <c r="A22" s="24" t="n">
         <v>18</v>
       </c>
-      <c r="B22" s="54" t="n"/>
-      <c r="C22" s="46" t="inlineStr">
+      <c r="B22" s="20" t="n"/>
+      <c r="C22" s="41" t="inlineStr">
         <is>
           <t>是否支持应用安装(仅标准系统涉及)</t>
         </is>
@@ -2001,7 +2018,7 @@
           <t>必选要求</t>
         </is>
       </c>
-      <c r="E22" s="43" t="inlineStr">
+      <c r="E22" s="39" t="inlineStr">
         <is>
           <t>1、检查测评中填写的是否支持应用安装信息与PCS自检表应用相关自检项的填写情况是否一致
 2、检查测评中填写的是否支持应用安装信息与测评中提供的XTS报告测试情况（是否执行相关用例）是否相符</t>
@@ -2009,14 +2026,14 @@
       </c>
       <c r="F22" s="29" t="n"/>
       <c r="G22" s="21" t="n"/>
-      <c r="H22" s="34" t="n"/>
-    </row>
-    <row r="23" ht="87" customHeight="1" s="51">
+      <c r="H22" s="32" t="n"/>
+    </row>
+    <row r="23" ht="87" customHeight="1" s="1">
       <c r="A23" s="24" t="n">
         <v>19</v>
       </c>
-      <c r="B23" s="54" t="n"/>
-      <c r="C23" s="46" t="inlineStr">
+      <c r="B23" s="20" t="n"/>
+      <c r="C23" s="41" t="inlineStr">
         <is>
           <t>是否带屏(仅标准系统涉及)</t>
         </is>
@@ -2026,7 +2043,7 @@
           <t>必选要求</t>
         </is>
       </c>
-      <c r="E23" s="43" t="inlineStr">
+      <c r="E23" s="39" t="inlineStr">
         <is>
           <t>1、检查测评中填写的是否带屏信息与PCS自检表屏幕相关自检项的填写情况是否一致
 2、检查测评中填写的是否带屏信息与测评中提供的XTS报告测试情况（是否执行相关用例）是否相符
@@ -2035,14 +2052,14 @@
       </c>
       <c r="F23" s="29" t="n"/>
       <c r="G23" s="21" t="n"/>
-      <c r="H23" s="34" t="n"/>
-    </row>
-    <row r="24" ht="87" customHeight="1" s="51">
+      <c r="H23" s="32" t="n"/>
+    </row>
+    <row r="24" ht="87" customHeight="1" s="1">
       <c r="A24" s="24" t="n">
         <v>20</v>
       </c>
-      <c r="B24" s="54" t="n"/>
-      <c r="C24" s="45" t="inlineStr">
+      <c r="B24" s="20" t="n"/>
+      <c r="C24" s="40" t="inlineStr">
         <is>
           <t>软件版本号</t>
         </is>
@@ -2052,7 +2069,7 @@
           <t>必选要求</t>
         </is>
       </c>
-      <c r="E24" s="43" t="inlineStr">
+      <c r="E24" s="39" t="inlineStr">
         <is>
           <t>1、用户可见的软件版本号，注意是整个系统的软件版本号而非OpenHarmony版本号。最多64字符。（即不允许带有OpenHarmony）
 2、测评中软件版本号、设备侧读取GetDisplayVersion()、XTS报告中DisplayVersion需保持一致</t>
@@ -2060,18 +2077,18 @@
       </c>
       <c r="F24" s="29" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✔</t>
         </is>
       </c>
       <c r="G24" s="21" t="n"/>
-      <c r="H24" s="34" t="n"/>
-    </row>
-    <row r="25" ht="69.59999999999999" customHeight="1" s="51">
+      <c r="H24" s="32" t="n"/>
+    </row>
+    <row r="25" ht="69.59999999999999" customHeight="1" s="1">
       <c r="A25" s="24" t="n">
         <v>21</v>
       </c>
-      <c r="B25" s="54" t="n"/>
-      <c r="C25" s="45" t="inlineStr">
+      <c r="B25" s="20" t="n"/>
+      <c r="C25" s="40" t="inlineStr">
         <is>
           <t>安全补丁标签</t>
         </is>
@@ -2081,27 +2098,31 @@
           <t>必选要求</t>
         </is>
       </c>
-      <c r="E25" s="43" t="inlineStr">
+      <c r="E25" s="39" t="inlineStr">
         <is>
           <t>1、安全补丁标签。标识当前OS的安全补丁级别。最多64字符。
 2、以补丁发布日期作为版本号，格式为"年/月/日"（即xxxx/xx/xx）。
 3、测评中安全补丁标签、设备侧读取GetSecurityPatchTag()、XTS报告中Security Patch需保持一致</t>
         </is>
       </c>
-      <c r="F25" s="29" t="n"/>
+      <c r="F25" s="29" t="inlineStr">
+        <is>
+          <t>✔</t>
+        </is>
+      </c>
       <c r="G25" s="21" t="n"/>
-      <c r="H25" s="32" t="inlineStr">
+      <c r="H25" s="31" t="inlineStr">
         <is>
           <t>驳回话术参考：1、测评信息，安全补丁标签“2024/9/1”与XTS报告中GetSecurityPatchTag()接口获取的“2024/09/01”不一致，需保持一致。</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="182" customHeight="1" s="51">
+    <row r="26" ht="182" customHeight="1" s="1">
       <c r="A26" s="24" t="n">
         <v>22</v>
       </c>
-      <c r="B26" s="54" t="n"/>
-      <c r="C26" s="45" t="inlineStr">
+      <c r="B26" s="20" t="n"/>
+      <c r="C26" s="40" t="inlineStr">
         <is>
           <t>版本id</t>
         </is>
@@ -2111,7 +2132,7 @@
           <t>必选要求</t>
         </is>
       </c>
-      <c r="E26" s="40" t="inlineStr">
+      <c r="E26" s="37" t="inlineStr">
         <is>
           <t>1、版本Id。由多个字段拼接而成：$(设备类型) + '/' + $(公司英文名简称) + '/' + $(品牌英文名称) + '/' + $(产品系列英文名称) + '/' + $( 操作系统及版本号 ) + '/' + $(型号) + '/' + $(内部软件子型号) + '/' + $(系统软件API level ) + '/' + $(差异版本号) + '/' + $(构建类型)，最多255字符。
 2、测评中版本Id、设备侧读取GetVersionId()、XTS报告中VersionId需保持一致
@@ -2121,18 +2142,18 @@
       </c>
       <c r="F26" s="29" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✔</t>
         </is>
       </c>
       <c r="G26" s="21" t="n"/>
-      <c r="H26" s="34" t="n"/>
-    </row>
-    <row r="27" ht="34.8" customHeight="1" s="51">
+      <c r="H26" s="32" t="n"/>
+    </row>
+    <row r="27" ht="34.8" customHeight="1" s="1">
       <c r="A27" s="24" t="n">
         <v>23</v>
       </c>
-      <c r="B27" s="53" t="n"/>
-      <c r="C27" s="45" t="inlineStr">
+      <c r="B27" s="19" t="n"/>
+      <c r="C27" s="40" t="inlineStr">
         <is>
           <t>版本Hash</t>
         </is>
@@ -2142,20 +2163,20 @@
           <t>必选要求</t>
         </is>
       </c>
-      <c r="E27" s="40" t="inlineStr">
+      <c r="E27" s="37" t="inlineStr">
         <is>
           <t>1、测评中版本Hash、设备侧 BuildRootHash、XTS报告中BuildRootHash均保持一致，其他无要求</t>
         </is>
       </c>
       <c r="F27" s="29" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✔</t>
         </is>
       </c>
       <c r="G27" s="21" t="n"/>
-      <c r="H27" s="34" t="n"/>
-    </row>
-    <row r="28" ht="139.2" customHeight="1" s="51">
+      <c r="H27" s="32" t="n"/>
+    </row>
+    <row r="28" ht="139.2" customHeight="1" s="1">
       <c r="A28" s="24" t="n">
         <v>24</v>
       </c>
@@ -2166,7 +2187,7 @@
 https://www.openharmony.cn/guide</t>
         </is>
       </c>
-      <c r="C28" s="48" t="inlineStr">
+      <c r="C28" s="42" t="inlineStr">
         <is>
           <t>基本信息描述</t>
         </is>
@@ -2176,7 +2197,7 @@
           <t>必选要求</t>
         </is>
       </c>
-      <c r="E28" s="49" t="inlineStr">
+      <c r="E28" s="43" t="inlineStr">
         <is>
           <t>1、检查是否与pcs自检表自检情况、XTS报告执行情况、豁免申请情况、测评中其他填写的信息是否相符一致。
 2、需要遵守《OpenHarmony兼容性标识使用指引 V1》的Powered by OpenHarmony传播描述规范相关规范，通过OpenHarmony兼容性测评的产品传播表达规范，规范描述表达仅限于以下三种：
@@ -2187,14 +2208,14 @@
       </c>
       <c r="F28" s="29" t="n"/>
       <c r="G28" s="21" t="n"/>
-      <c r="H28" s="34" t="n"/>
-    </row>
-    <row r="29" ht="168" customHeight="1" s="51">
+      <c r="H28" s="32" t="n"/>
+    </row>
+    <row r="29" ht="168" customHeight="1" s="1">
       <c r="A29" s="24" t="n">
         <v>25</v>
       </c>
-      <c r="B29" s="53" t="n"/>
-      <c r="C29" s="48" t="inlineStr">
+      <c r="B29" s="19" t="n"/>
+      <c r="C29" s="42" t="inlineStr">
         <is>
           <t>外观图</t>
         </is>
@@ -2204,7 +2225,7 @@
           <t>必选要求</t>
         </is>
       </c>
-      <c r="E29" s="50" t="inlineStr">
+      <c r="E29" s="44" t="inlineStr">
         <is>
           <t>1、商用设备
 图片尺寸：400*400
@@ -2216,7 +2237,7 @@
       </c>
       <c r="F29" s="29" t="n"/>
       <c r="G29" s="29" t="n"/>
-      <c r="H29" s="32" t="inlineStr">
+      <c r="H29" s="31" t="inlineStr">
         <is>
           <t>如果样机体积较大或者成本过高，可以发非整机投递申请给工作组邮箱compatibility@mail.openharmony.io，
 样机投递：
@@ -2228,7 +2249,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="213" customHeight="1" s="51">
+    <row r="30" ht="213" customHeight="1" s="1">
       <c r="A30" s="24" t="n">
         <v>26</v>
       </c>
@@ -2263,18 +2284,18 @@
       </c>
       <c r="F30" s="29" t="n"/>
       <c r="G30" s="21" t="n"/>
-      <c r="H30" s="32" t="n"/>
-    </row>
-    <row r="31" ht="33" customHeight="1" s="51">
+      <c r="H30" s="31" t="n"/>
+    </row>
+    <row r="31" ht="33" customHeight="1" s="1">
       <c r="A31" s="24" t="n">
         <v>27</v>
       </c>
-      <c r="B31" s="37" t="inlineStr">
+      <c r="B31" s="34" t="inlineStr">
         <is>
           <t>其他要求</t>
         </is>
       </c>
-      <c r="C31" s="37" t="inlineStr">
+      <c r="C31" s="34" t="inlineStr">
         <is>
           <t>归档</t>
         </is>
@@ -2284,34 +2305,34 @@
           <t>必选要求</t>
         </is>
       </c>
-      <c r="E31" s="38" t="inlineStr">
+      <c r="E31" s="35" t="inlineStr">
         <is>
           <t>XTS测试报告、Checklist填写涉及信息需保证真实有效，不允许存在业务造假或其他质量重大问题</t>
         </is>
       </c>
       <c r="F31" s="29" t="n"/>
-      <c r="G31" s="41" t="n"/>
-      <c r="H31" s="34" t="n"/>
+      <c r="G31" s="38" t="n"/>
+      <c r="H31" s="32" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="24" t="n">
         <v>28</v>
       </c>
-      <c r="B32" s="53" t="n"/>
-      <c r="C32" s="53" t="n"/>
+      <c r="B32" s="19" t="n"/>
+      <c r="C32" s="19" t="n"/>
       <c r="D32" s="27" t="inlineStr">
         <is>
           <t>必选要求</t>
         </is>
       </c>
-      <c r="E32" s="38" t="inlineStr">
+      <c r="E32" s="35" t="inlineStr">
         <is>
           <t>合作中心测试的XTS报告、Checklist，需单独归档</t>
         </is>
       </c>
       <c r="F32" s="29" t="n"/>
-      <c r="G32" s="41" t="n"/>
-      <c r="H32" s="34" t="n"/>
+      <c r="G32" s="38" t="n"/>
+      <c r="H32" s="32" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="13">
@@ -2356,117 +2377,117 @@
   <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
-    <col width="18.1296296296296" customWidth="1" style="51" min="1" max="1"/>
-    <col width="19.6018518518519" customWidth="1" style="51" min="2" max="2"/>
-    <col width="8.731481481481479" customWidth="1" style="51" min="3" max="3"/>
-    <col width="21.2685185185185" customWidth="1" style="51" min="4" max="4"/>
-    <col width="17" customWidth="1" style="51" min="5" max="5"/>
-    <col width="27" customWidth="1" style="51" min="6" max="6"/>
-    <col width="22.3981481481481" customWidth="1" style="51" min="8" max="8"/>
-    <col width="35.462962962963" customWidth="1" style="51" min="9" max="9"/>
+    <col width="18.1296296296296" customWidth="1" style="1" min="1" max="1"/>
+    <col width="19.6018518518519" customWidth="1" style="1" min="2" max="2"/>
+    <col width="8.731481481481479" customWidth="1" style="1" min="3" max="3"/>
+    <col width="21.2685185185185" customWidth="1" style="1" min="4" max="4"/>
+    <col width="17" customWidth="1" style="1" min="5" max="5"/>
+    <col width="27" customWidth="1" style="1" min="6" max="6"/>
+    <col width="22.3981481481481" customWidth="1" style="1" min="8" max="8"/>
+    <col width="35.462962962963" customWidth="1" style="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="19.2" customHeight="1" s="51">
-      <c r="A1" s="1" t="n"/>
-    </row>
-    <row r="2" ht="16.35" customHeight="1" s="51">
-      <c r="A2" s="2" t="n"/>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
-      <c r="I2" s="3" t="n"/>
-    </row>
-    <row r="3" ht="15.15" customHeight="1" s="51">
-      <c r="A3" s="4" t="n"/>
-      <c r="B3" s="4" t="n"/>
-      <c r="C3" s="4" t="n"/>
-      <c r="D3" s="4" t="n"/>
-      <c r="E3" s="4" t="n"/>
-      <c r="F3" s="4" t="n"/>
-      <c r="G3" s="4" t="n"/>
-      <c r="H3" s="4" t="n"/>
-      <c r="I3" s="4" t="n"/>
-    </row>
-    <row r="4" ht="15.15" customHeight="1" s="51">
-      <c r="A4" s="5" t="n"/>
-      <c r="B4" s="5" t="n"/>
-      <c r="C4" s="5" t="n"/>
-      <c r="D4" s="5" t="n"/>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="5" t="n"/>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="5" t="n"/>
-      <c r="I4" s="5" t="n"/>
-    </row>
-    <row r="5" ht="15.15" customHeight="1" s="51">
-      <c r="A5" s="6" t="n"/>
-      <c r="B5" s="6" t="n"/>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="6" t="n"/>
-      <c r="G5" s="6" t="n"/>
-      <c r="H5" s="6" t="n"/>
-      <c r="I5" s="6" t="n"/>
-    </row>
-    <row r="6" ht="15.75" customHeight="1" s="51">
-      <c r="A6" s="5" t="n"/>
-      <c r="B6" s="5" t="n"/>
-      <c r="C6" s="5" t="n"/>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="5" t="n"/>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="5" t="n"/>
-      <c r="H6" s="5" t="n"/>
-      <c r="I6" s="7" t="n"/>
-    </row>
-    <row r="7" ht="15.75" customHeight="1" s="51">
-      <c r="A7" s="6" t="n"/>
-      <c r="B7" s="6" t="n"/>
-      <c r="C7" s="6" t="n"/>
-      <c r="D7" s="6" t="n"/>
-      <c r="E7" s="6" t="n"/>
-      <c r="F7" s="6" t="n"/>
-      <c r="G7" s="6" t="n"/>
-      <c r="H7" s="6" t="n"/>
-      <c r="I7" s="8" t="n"/>
-    </row>
-    <row r="8" ht="15.75" customHeight="1" s="51">
-      <c r="A8" s="5" t="n"/>
-      <c r="B8" s="5" t="n"/>
-      <c r="C8" s="5" t="n"/>
-      <c r="D8" s="5" t="n"/>
-      <c r="E8" s="5" t="n"/>
-      <c r="F8" s="5" t="n"/>
-      <c r="G8" s="5" t="n"/>
-      <c r="H8" s="5" t="n"/>
-      <c r="I8" s="7" t="n"/>
-    </row>
-    <row r="9" ht="15.15" customHeight="1" s="51">
-      <c r="A9" s="6" t="n"/>
-      <c r="B9" s="6" t="n"/>
-      <c r="C9" s="6" t="n"/>
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="6" t="n"/>
-      <c r="F9" s="6" t="n"/>
-      <c r="G9" s="6" t="n"/>
-      <c r="H9" s="6" t="n"/>
-      <c r="I9" s="6" t="n"/>
-    </row>
-    <row r="10" ht="15.75" customHeight="1" s="51">
-      <c r="A10" s="9" t="n"/>
-      <c r="B10" s="9" t="n"/>
-      <c r="C10" s="9" t="n"/>
-      <c r="D10" s="9" t="n"/>
-      <c r="E10" s="9" t="n"/>
-      <c r="F10" s="9" t="n"/>
-      <c r="G10" s="9" t="n"/>
-      <c r="H10" s="9" t="n"/>
-      <c r="I10" s="10" t="n"/>
+    <row r="1" ht="19.2" customHeight="1" s="1">
+      <c r="A1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="16.35" customHeight="1" s="1">
+      <c r="A2" s="3" t="n"/>
+      <c r="B2" s="3" t="n"/>
+      <c r="C2" s="3" t="n"/>
+      <c r="D2" s="3" t="n"/>
+      <c r="E2" s="3" t="n"/>
+      <c r="F2" s="3" t="n"/>
+      <c r="G2" s="3" t="n"/>
+      <c r="H2" s="3" t="n"/>
+      <c r="I2" s="4" t="n"/>
+    </row>
+    <row r="3" ht="15.15" customHeight="1" s="1">
+      <c r="A3" s="5" t="n"/>
+      <c r="B3" s="5" t="n"/>
+      <c r="C3" s="5" t="n"/>
+      <c r="D3" s="5" t="n"/>
+      <c r="E3" s="5" t="n"/>
+      <c r="F3" s="5" t="n"/>
+      <c r="G3" s="5" t="n"/>
+      <c r="H3" s="5" t="n"/>
+      <c r="I3" s="5" t="n"/>
+    </row>
+    <row r="4" ht="15.15" customHeight="1" s="1">
+      <c r="A4" s="6" t="n"/>
+      <c r="B4" s="6" t="n"/>
+      <c r="C4" s="6" t="n"/>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="6" t="n"/>
+      <c r="G4" s="6" t="n"/>
+      <c r="H4" s="6" t="n"/>
+      <c r="I4" s="6" t="n"/>
+    </row>
+    <row r="5" ht="15.15" customHeight="1" s="1">
+      <c r="A5" s="7" t="n"/>
+      <c r="B5" s="7" t="n"/>
+      <c r="C5" s="7" t="n"/>
+      <c r="D5" s="7" t="n"/>
+      <c r="E5" s="7" t="n"/>
+      <c r="F5" s="7" t="n"/>
+      <c r="G5" s="7" t="n"/>
+      <c r="H5" s="7" t="n"/>
+      <c r="I5" s="7" t="n"/>
+    </row>
+    <row r="6" ht="15.75" customHeight="1" s="1">
+      <c r="A6" s="6" t="n"/>
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="6" t="n"/>
+      <c r="D6" s="6" t="n"/>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="6" t="n"/>
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="6" t="n"/>
+      <c r="I6" s="8" t="n"/>
+    </row>
+    <row r="7" ht="15.75" customHeight="1" s="1">
+      <c r="A7" s="7" t="n"/>
+      <c r="B7" s="7" t="n"/>
+      <c r="C7" s="7" t="n"/>
+      <c r="D7" s="7" t="n"/>
+      <c r="E7" s="7" t="n"/>
+      <c r="F7" s="7" t="n"/>
+      <c r="G7" s="7" t="n"/>
+      <c r="H7" s="7" t="n"/>
+      <c r="I7" s="9" t="n"/>
+    </row>
+    <row r="8" ht="15.75" customHeight="1" s="1">
+      <c r="A8" s="6" t="n"/>
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="6" t="n"/>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="6" t="n"/>
+      <c r="F8" s="6" t="n"/>
+      <c r="G8" s="6" t="n"/>
+      <c r="H8" s="6" t="n"/>
+      <c r="I8" s="8" t="n"/>
+    </row>
+    <row r="9" ht="15.15" customHeight="1" s="1">
+      <c r="A9" s="7" t="n"/>
+      <c r="B9" s="7" t="n"/>
+      <c r="C9" s="7" t="n"/>
+      <c r="D9" s="7" t="n"/>
+      <c r="E9" s="7" t="n"/>
+      <c r="F9" s="7" t="n"/>
+      <c r="G9" s="7" t="n"/>
+      <c r="H9" s="7" t="n"/>
+      <c r="I9" s="7" t="n"/>
+    </row>
+    <row r="10" ht="15.75" customHeight="1" s="1">
+      <c r="A10" s="10" t="n"/>
+      <c r="B10" s="10" t="n"/>
+      <c r="C10" s="10" t="n"/>
+      <c r="D10" s="10" t="n"/>
+      <c r="E10" s="10" t="n"/>
+      <c r="F10" s="10" t="n"/>
+      <c r="G10" s="10" t="n"/>
+      <c r="H10" s="10" t="n"/>
+      <c r="I10" s="11" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>